<commit_message>
docs(w15): add stage 4f local input preflight
</commit_message>
<xml_diff>
--- a/docs/examples/intelligence-stage4f-data-request/intelligence-stage4f-data-template.xlsx
+++ b/docs/examples/intelligence-stage4f-data-request/intelligence-stage4f-data-template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R7eacb8d152994253"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observações" sheetId="2" r:id="Ra0252734a9644f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa TAG" sheetId="3" r:id="Rb960727415664aef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coortes" sheetId="4" r:id="Rf3964f600aee45fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critérios" sheetId="5" r:id="R1d048c2cda78430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicionário" sheetId="6" r:id="Rc595e171648943d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R3071ff4152824d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observações" sheetId="2" r:id="R1deeb61670064234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa TAG" sheetId="3" r:id="R670eb52d289743f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coortes" sheetId="4" r:id="R36f4fbdf9c3d4815"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critérios" sheetId="5" r:id="R560ad01684664b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicionário" sheetId="6" r:id="R67785c586ca14022"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -713,7 +713,7 @@
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Modelo em branco para preparar a avaliação. Não contém histórico real nem define limites numéricos.</x:v>
+        <x:v>Modelo em branco para preparar a avaliação. Não contém histórico real. Use o plano aceito do Stage 4F para metas e regras; a análise ainda depende de uma coorte autorizada.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -826,7 +826,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>Defina denominadores, janelas e metas aceitas. Não use limites pré-preenchidos.</x:v>
+        <x:v>Use as metas e regras de avaliação do plano aceito do Stage 4F. Registre somente os dados específicos e a autorização desta coleta.</x:v>
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2" t="str">
@@ -880,7 +880,7 @@
         <x:v>Estado</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>4F continua NOT READY até haver dados representativos autorizados e critérios aceitos.</x:v>
+        <x:v>4F continua NOT READY até que dados representativos autorizados sejam avaliados contra o plano aceito.</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2" t="str">
@@ -909,10 +909,10 @@
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>Sem meta presumida</x:v>
+        <x:v>Metas no plano aceito</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>Não há limite de falso alarme, sensibilidade, tamanho mínimo ou limiar pré-preenchido.</x:v>
+        <x:v>O plano define as metas iniciais. Suficiência, calibração e limiar do método ainda dependem de dados representativos autorizados.</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
       <x:c r="D17" s="2" t="str">
@@ -1184,7 +1184,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb796ec4651a41d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re02f721f24ef4310"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1354,7 +1354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4adb0c8525548a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66a9b7a16225459b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd590a7b100b4193"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc199c57a87554c10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1560,7 +1560,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>Critérios que o Product Owner precisa definir</x:v>
+        <x:v>Critérios aceitos e pendências da coleta</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -1573,7 +1573,7 @@
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>As respostas e metas permanecem em branco. Nenhum limite estatístico é presumido por este modelo.</x:v>
+        <x:v>As metas e regras seguem o plano aceito do Stage 4F. Não defina novamente limites numéricos; registre apenas dados e evidências específicos da coorte.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -1606,10 +1606,10 @@
         <x:v>Definição necessária</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Resposta do Product Owner</x:v>
+        <x:v>Registro da coleta/referência</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Meta/condição aceita</x:v>
+        <x:v>Plano aceito/condição específica</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
         <x:v>População, unidade e janela</x:v>
@@ -1640,7 +1640,7 @@
       <x:c r="G6" s="33" t="str"/>
       <x:c r="H6" s="33" t="str"/>
       <x:c r="I6" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Coorte pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
@@ -1659,7 +1659,7 @@
       <x:c r="G7" s="33" t="str"/>
       <x:c r="H7" s="33" t="str"/>
       <x:c r="I7" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Regra aceita</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
@@ -1678,7 +1678,7 @@
       <x:c r="G8" s="33" t="str"/>
       <x:c r="H8" s="33" t="str"/>
       <x:c r="I8" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Regra aceita; medir</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
@@ -1697,7 +1697,7 @@
       <x:c r="G9" s="33" t="str"/>
       <x:c r="H9" s="33" t="str"/>
       <x:c r="I9" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Meta aceita; avaliar</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
@@ -1716,7 +1716,7 @@
       <x:c r="G10" s="33" t="str"/>
       <x:c r="H10" s="33" t="str"/>
       <x:c r="I10" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Cenários definidos</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
@@ -1735,7 +1735,7 @@
       <x:c r="G11" s="33" t="str"/>
       <x:c r="H11" s="33" t="str"/>
       <x:c r="I11" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Meta aceita; medir</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
@@ -1754,7 +1754,7 @@
       <x:c r="G12" s="33" t="str"/>
       <x:c r="H12" s="33" t="str"/>
       <x:c r="I12" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Regra aceita; manifesto pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -1773,7 +1773,7 @@
       <x:c r="G13" s="33" t="str"/>
       <x:c r="H13" s="33" t="str"/>
       <x:c r="I13" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Piso definido; avaliar</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -1792,7 +1792,7 @@
       <x:c r="G14" s="33" t="str"/>
       <x:c r="H14" s="33" t="str"/>
       <x:c r="I14" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Regra aceita; evidência pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
@@ -1803,7 +1803,7 @@
         <x:v>Uso e retenção</x:v>
       </x:c>
       <x:c r="C15" s="32" t="str">
-        <x:v>Responsável pelos dados, finalidade, ambiente autorizado, pessoas permitidas, retenção e método/data de expurgo.</x:v>
+        <x:v>Responsável pelos dados, finalidade autorizada, armazenamento e acessos permitidos; aplicar os limites de retenção/expurgo do plano.</x:v>
       </x:c>
       <x:c r="D15" s="33" t="str"/>
       <x:c r="E15" s="33" t="str"/>
@@ -1811,7 +1811,7 @@
       <x:c r="G15" s="33" t="str"/>
       <x:c r="H15" s="33" t="str"/>
       <x:c r="I15" s="36" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Retenção definida; autorização pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -1819,10 +1819,10 @@
         <x:v>ACCEPT-01</x:v>
       </x:c>
       <x:c r="B16" s="38" t="str">
-        <x:v>Aceite do Product Owner</x:v>
+        <x:v>Plano aceito e autorização da coorte</x:v>
       </x:c>
       <x:c r="C16" s="38" t="str">
-        <x:v>Aprovação explícita do escopo, das métricas/limites e da autorização de uso antes de liberar a implementação 4F.</x:v>
+        <x:v>Metas e regras de avaliação definidas no plano aceito; autorização específica da coorte e confirmação de proveniência ainda necessárias.</x:v>
       </x:c>
       <x:c r="D16" s="39" t="str"/>
       <x:c r="E16" s="39" t="str"/>
@@ -1830,7 +1830,7 @@
       <x:c r="G16" s="39" t="str"/>
       <x:c r="H16" s="39" t="str"/>
       <x:c r="I16" s="40" t="str">
-        <x:v>Aguardando definição</x:v>
+        <x:v>Plano aceito; autorização pendente</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2100,7 +2100,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff8f59bb1bd04cde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72b9b8707fb64e98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2622,8 +2622,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3596d32165d48a5"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7fcb22baafa4fb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41dcb76f434a4436"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba4b0cd71a194002"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>